<commit_message>
feat: add new dataset
</commit_message>
<xml_diff>
--- a/data/proteomics/omics_Francesca_scale.xlsx
+++ b/data/proteomics/omics_Francesca_scale.xlsx
@@ -36711,9 +36711,7 @@
           <t>YMR142C</t>
         </is>
       </c>
-      <c r="C1910" t="n">
-        <v>0.008132535259730709</v>
-      </c>
+      <c r="C1910" t="inlineStr"/>
       <c r="D1910" t="n">
         <v>0.0003537504799997783</v>
       </c>

</xml_diff>